<commit_message>
Deployed a2ca32c33 to run-update with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/run-update/catalog_summary.xlsx
+++ b/run-update/catalog_summary.xlsx
@@ -1614,11 +1614,11 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="V11" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr"/>
@@ -1850,12 +1850,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
+          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
+          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1865,7 +1865,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
+          <t>Kelp forest communities along an otter gradient</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1883,12 +1883,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>underDevelopment</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Simon Fraser University</t>
         </is>
       </c>
       <c r="N14" t="n">
@@ -1911,12 +1911,12 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -1924,14 +1924,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>10.21966/nmds-rx42</t>
-        </is>
-      </c>
+      <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXp1R01BNWFYV0RkUEY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXlMbjJYUlpvZFpITks</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -1941,25 +1937,15 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2024-07-23</t>
         </is>
       </c>
       <c r="V14" t="n">
-        <v>3</v>
-      </c>
-      <c r="W14" t="n">
-        <v>0</v>
-      </c>
-      <c r="X14" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="Y14" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr"/>
+      <c r="Y14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1967,12 +1953,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>f5d51d99-ce24-4713-a317-7927dd283f1a</t>
+          <t>0d9ca9c8-95b0-48db-87b9-7db8af77363e</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ca-cioos_af65bf72-27af-4747-8911-ab05591762ac</t>
+          <t>ca-cioos_ab901b46-43f6-4044-b0c3-b5fd825622f4</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1982,7 +1968,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Kelp forest communities along an otter gradient</t>
+          <t>World View 2 Imagery - Coverage of three regions of the BC Central Coast - Summer 2014, 2015, &amp; 2016</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2000,12 +1986,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>underDevelopment</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2020,7 +2006,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Simon Fraser University</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N15" t="n">
@@ -2028,12 +2014,12 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.770751953125, 51.33404377878941], [-127.74902343749999, 51.33404377878941], [-127.74902343749999, 52.19077237113535], [-128.770751953125, 52.19077237113535], [-128.770751953125, 51.33404377878941]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.61145019531247, 51.61801654877371], [-127.91931152343746, 51.61801654877371], [-127.91931152343746, 52.11325243469631], [-128.61145019531247, 52.11325243469631], [-128.61145019531247, 51.61801654877371]]]}</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -2041,10 +2027,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr"/>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>10.21966/nmds-rx42</t>
+        </is>
+      </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXlMbjJYUlpvZFpITks</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXp1R01BNWFYV0RkUEY</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -2054,15 +2044,25 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V15" t="n">
-        <v>5</v>
-      </c>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
-      <c r="Y15" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="W15" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -5013,7 +5013,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Nereocystis kelp canopy productivity data from BC Central Coast, v1.2.0</t>
+          <t>Nereocystis kelp canopy productivity data from BC Central Coast</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -5089,12 +5089,10 @@
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
-        </is>
-      </c>
-      <c r="V42" t="n">
-        <v>7</v>
-      </c>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr"/>
       <c r="W42" t="n">
         <v>1</v>
       </c>
@@ -6574,12 +6572,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>9b7adebb-5027-486a-8ed1-f97b5353a480</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ca-cioos_6ebe47c3-6d59-4cb2-a7ba-111698445d8d</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -6589,7 +6587,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Bald eagles as vectors of marine nutrients – Central Coast Islands (100 Islands study area) – May – July 2017</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -6607,7 +6605,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>100 Islands</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -6627,15 +6625,15 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.58323147, 51.38160352], [-127.80979387, 51.38160352], [-127.80979387, 52.09997599], [-128.58323147, 52.09997599], [-128.58323147, 51.38160352]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
@@ -6645,13 +6643,17 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>other, nutrients</t>
-        </is>
-      </c>
-      <c r="R56" t="inlineStr"/>
+          <t>other, inorganicCarbon</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>10.21966/zxzr-e472</t>
+        </is>
+      </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxkcndoNFQ4T2xyZWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T56" t="inlineStr">
@@ -6661,15 +6663,23 @@
       </c>
       <c r="U56" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="V56" t="n">
-        <v>1</v>
-      </c>
-      <c r="W56" t="inlineStr"/>
-      <c r="X56" t="inlineStr"/>
-      <c r="Y56" t="inlineStr"/>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr"/>
+      <c r="W56" t="n">
+        <v>0</v>
+      </c>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -6677,12 +6687,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>9b7adebb-5027-486a-8ed1-f97b5353a480</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6ebe47c3-6d59-4cb2-a7ba-111698445d8d</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -6692,7 +6702,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Bald eagles as vectors of marine nutrients – Central Coast Islands (100 Islands study area) – May – July 2017</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -6710,7 +6720,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>100 Islands</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -6730,61 +6740,49 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N57" t="n">
+        <v>2</v>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.58323147, 51.38160352], [-127.80979387, 51.38160352], [-127.80979387, 52.09997599], [-128.58323147, 52.09997599], [-128.58323147, 51.38160352]]]}</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>other, nutrients</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxkcndoNFQ4T2xyZWI</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>2022-01-24</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="V57" t="n">
         <v>1</v>
       </c>
-      <c r="O57" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
-        </is>
-      </c>
-      <c r="P57" t="inlineStr">
-        <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q57" t="inlineStr">
-        <is>
-          <t>other, inorganicCarbon</t>
-        </is>
-      </c>
-      <c r="R57" t="inlineStr">
-        <is>
-          <t>10.21966/zxzr-e472</t>
-        </is>
-      </c>
-      <c r="S57" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
-        </is>
-      </c>
-      <c r="T57" t="inlineStr">
-        <is>
-          <t>2022-01-24</t>
-        </is>
-      </c>
-      <c r="U57" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="V57" t="inlineStr"/>
-      <c r="W57" t="n">
-        <v>0</v>
-      </c>
-      <c r="X57" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="Y57" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="W57" t="inlineStr"/>
+      <c r="X57" t="inlineStr"/>
+      <c r="Y57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -6909,12 +6907,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>9e4a38d6-eb29-44a8-b495-c56ce74a227c</t>
+          <t>dd5c8784-c292-4f68-bc3d-a460adb8cdbf</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ca-cioos_c113d7a8-6a46-46fc-b49c-a4e69afedfbc</t>
+          <t>ca-cioos_b4cac70e-a6fa-4d77-8fdb-1d3612006bc4</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -6924,7 +6922,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Hakai Institute’s Burke-o-Lator TCO2/pCO2 Analyzer Discrete Sample Analysis Protocols</t>
+          <t>Pacific Northwest Eelgrass Sediment Carbon Data</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -6942,7 +6940,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -6966,31 +6964,31 @@
         </is>
       </c>
       <c r="N59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.200851030026, 47.5931373865871], [-133.329762644444, 58.3685518859093], [-138.778981394444, 57.2923559868765], [-128.407887644444, 50.1363698995369], [-122.519210405026, 46.8770323398551], [-121.200851030026, 47.5931373865871]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-143.1666738, 39.75452039], [-118.41060343, 39.75452039], [-118.41060343, 59.04838928], [-143.1666738, 59.04838928], [-143.1666738, 39.75452039]]]}</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>[{'max': '50.15267028510888', 'min': '50.15091039641325'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, seagrassCoverAndComposition</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>10.21966/1.521066</t>
+          <t>10.21966/20SJ-J017</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUQyQ3F1WFBEZ2FkTnI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVlYNnVCWW5yQ3RrUkM</t>
         </is>
       </c>
       <c r="T59" t="inlineStr">
@@ -7000,21 +6998,23 @@
       </c>
       <c r="U59" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V59" t="inlineStr"/>
+          <t>2025-04-23</t>
+        </is>
+      </c>
+      <c r="V59" t="n">
+        <v>8</v>
+      </c>
       <c r="W59" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X59" t="inlineStr">
         <is>
-          <t>[{'year': '2024', 'total': 1}, {'year': '2025', 'total': 2}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="Y59" t="inlineStr">
         <is>
-          <t>[{'relationship': 'citations', 'id': '10.21966/k1xg-6920', 'type': 'dois', 'status_code': 200, 'url': 'https://catalogue.hakai.org/dataset/ca-cioos_355467ad-104d-40a6-b06e-52a67bfe247e'}, {'relationship': 'citations', 'id': '10.1002/eap.70058', 'type': 'dois', 'status_code': 403, 'url': 'https://esajournals.onlinelibrary.wiley.com/doi/10.1002/eap.70058'}, {'relationship': 'citations', 'id': '10.1002/edn3.70158', 'type': 'dois', 'status_code': 403, 'url': 'https://onlinelibrary.wiley.com/doi/10.1002/edn3.70158'}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -7024,12 +7024,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
+          <t>9e4a38d6-eb29-44a8-b495-c56ce74a227c</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>ca-cioos_d200376b-7dd8-4778-b3f5-379243bf93b8</t>
+          <t>ca-cioos_c113d7a8-6a46-46fc-b49c-a4e69afedfbc</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -7039,7 +7039,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>High-resolution record of surface water pH at Sentry Shoal in the Northern Strait of Georgia</t>
+          <t>Hakai Institute’s Burke-o-Lator TCO2/pCO2 Analyzer Discrete Sample Analysis Protocols</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -7081,31 +7081,31 @@
         </is>
       </c>
       <c r="N60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.9855, 49.9066], [-124.9854, 49.9066], [-124.9854, 49.9067], [-124.9855, 49.9067], [-124.9855, 49.9066]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.200851030026, 47.5931373865871], [-133.329762644444, 58.3685518859093], [-138.778981394444, 57.2923559868765], [-128.407887644444, 50.1363698995369], [-122.519210405026, 46.8770323398551], [-121.200851030026, 47.5931373865871]]]}</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.15267028510888', 'min': '50.15091039641325'}]</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>10.21966/1.715693</t>
+          <t>10.21966/1.521066</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUlpdWJIYjdIVDZJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUQyQ3F1WFBEZ2FkTnI</t>
         </is>
       </c>
       <c r="T60" t="inlineStr">
@@ -7118,20 +7118,18 @@
           <t>2024-07-24</t>
         </is>
       </c>
-      <c r="V60" t="n">
-        <v>1</v>
-      </c>
+      <c r="V60" t="inlineStr"/>
       <c r="W60" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="X60" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2024', 'total': 1}, {'year': '2025', 'total': 2}]</t>
         </is>
       </c>
       <c r="Y60" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'relationship': 'citations', 'id': '10.21966/k1xg-6920', 'type': 'dois', 'status_code': 200, 'url': 'https://catalogue.hakai.org/dataset/ca-cioos_355467ad-104d-40a6-b06e-52a67bfe247e'}, {'relationship': 'citations', 'id': '10.1002/eap.70058', 'type': 'dois', 'status_code': 403, 'url': 'https://esajournals.onlinelibrary.wiley.com/doi/10.1002/eap.70058'}, {'relationship': 'citations', 'id': '10.1002/edn3.70158', 'type': 'dois', 'status_code': 403, 'url': 'https://onlinelibrary.wiley.com/doi/10.1002/edn3.70158'}]</t>
         </is>
       </c>
     </row>
@@ -7141,12 +7139,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>24c3b914-33d7-4267-a1aa-8ce7523b296d</t>
+          <t>1f798a06-9c01-4025-93c6-b1a9f8ce6832</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ca-cioos_dc50a22a-44c0-478c-aa19-a46343bc764a</t>
+          <t>ca-cioos_d200376b-7dd8-4778-b3f5-379243bf93b8</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -7156,7 +7154,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Barnacle Dynamics: Point Intercept Surveys - BC Central Coast - 2019</t>
+          <t>High-resolution record of surface water pH at Sentry Shoal in the Northern Strait of Georgia</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -7174,7 +7172,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -7202,7 +7200,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.1518199, 51.64582999], [-128.12195082, 51.64582999], [-128.12195082, 51.66861942], [-128.1518199, 51.66861942], [-128.1518199, 51.64582999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.9855, 49.9066], [-124.9854, 49.9066], [-124.9854, 49.9067], [-124.9855, 49.9067], [-124.9855, 49.9066]]]}</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
@@ -7217,12 +7215,12 @@
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>10.21966/m8kp-gy81</t>
+          <t>10.21966/1.715693</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUFaZGRYOURGWVg5UzA</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUlpdWJIYjdIVDZJWTk</t>
         </is>
       </c>
       <c r="T61" t="inlineStr">
@@ -7232,10 +7230,12 @@
       </c>
       <c r="U61" t="inlineStr">
         <is>
-          <t>2024-08-02</t>
-        </is>
-      </c>
-      <c r="V61" t="inlineStr"/>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V61" t="n">
+        <v>1</v>
+      </c>
       <c r="W61" t="n">
         <v>0</v>
       </c>
@@ -7256,12 +7256,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>d8d3f510-8d7c-4b51-ba80-f7a77244eb4e</t>
+          <t>24c3b914-33d7-4267-a1aa-8ce7523b296d</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>ca-cioos_f00b9c87-190e-4b89-a864-7c012b989e49</t>
+          <t>ca-cioos_dc50a22a-44c0-478c-aa19-a46343bc764a</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -7271,7 +7271,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>High-resolution record of surface seawater CO2 content from December 2014 to April 2016 collected in Hyacinthe Bay, British Columbia, Canada. Version 1.0.</t>
+          <t>Barnacle Dynamics: Point Intercept Surveys - BC Central Coast - 2019</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -7289,7 +7289,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -7313,31 +7313,31 @@
         </is>
       </c>
       <c r="N62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.2229619026184, 50.116395452024676], [-125.22092342376709, 50.116395452024676], [-125.22092342376709, 50.11764753238538], [-125.2229619026184, 50.11764753238538], [-125.2229619026184, 50.116395452024676]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.1518199, 51.64582999], [-128.12195082, 51.64582999], [-128.12195082, 51.66861942], [-128.1518199, 51.66861942], [-128.1518199, 51.64582999]]]}</t>
         </is>
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>[{'max': '1.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>10.21966/1.437736</t>
+          <t>10.21966/m8kp-gy81</t>
         </is>
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXg3Yk10WFU2UGRwYkY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUFaZGRYOURGWVg5UzA</t>
         </is>
       </c>
       <c r="T62" t="inlineStr">
@@ -7347,12 +7347,10 @@
       </c>
       <c r="U62" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V62" t="n">
-        <v>3</v>
-      </c>
+          <t>2024-08-02</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr"/>
       <c r="W62" t="n">
         <v>0</v>
       </c>
@@ -7373,12 +7371,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ad032cd1-86cc-47cc-ac01-fce09e4cf8d9</t>
+          <t>d8d3f510-8d7c-4b51-ba80-f7a77244eb4e</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>ca-cioos_fcb4dfb6-606b-4b4b-bdcb-90f3f480fc33</t>
+          <t>ca-cioos_f00b9c87-190e-4b89-a864-7c012b989e49</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -7388,7 +7386,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Data on invasion of Calvert Island by Orthione griffenis</t>
+          <t>High-resolution record of surface seawater CO2 content from December 2014 to April 2016 collected in Hyacinthe Bay, British Columbia, Canada. Version 1.0.</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -7404,7 +7402,11 @@
       <c r="H63" t="b">
         <v>0</v>
       </c>
-      <c r="I63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Oceanography</t>
+        </is>
+      </c>
       <c r="J63" t="inlineStr">
         <is>
           <t>completed</t>
@@ -7426,31 +7428,31 @@
         </is>
       </c>
       <c r="N63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.17334953, 51.61670267], [-127.92753044, 51.61670267], [-127.92753044, 51.73677458], [-128.17334953, 51.73677458], [-128.17334953, 51.61670267]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.2229619026184, 50.116395452024676], [-125.22092342376709, 50.116395452024676], [-125.22092342376709, 50.11764753238538], [-125.2229619026184, 50.11764753238538], [-125.2229619026184, 50.116395452024676]]]}</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>10.21966/kddh-gj22</t>
+          <t>10.21966/1.437736</t>
         </is>
       </c>
       <c r="S63" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWpwT0Z6RlAySHp6cU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXg3Yk10WFU2UGRwYkY</t>
         </is>
       </c>
       <c r="T63" t="inlineStr">
@@ -7464,7 +7466,7 @@
         </is>
       </c>
       <c r="V63" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="W63" t="n">
         <v>0</v>
@@ -7486,12 +7488,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
+          <t>ad032cd1-86cc-47cc-ac01-fce09e4cf8d9</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>ca-cioos_41b0137d-6ac0-407d-a550-dd375475b2b0</t>
+          <t>ca-cioos_fcb4dfb6-606b-4b4b-bdcb-90f3f480fc33</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -7501,7 +7503,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Seafloor Observatory in Hyacinthe Bay, Quadra Island, British Columbia, Canada (Provisional)</t>
+          <t>Data on invasion of Calvert Island by Orthione griffenis</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -7517,14 +7519,10 @@
       <c r="H64" t="b">
         <v>0</v>
       </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>Oceanography</t>
-        </is>
-      </c>
+      <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -7547,41 +7545,55 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-125.22003, 50.11736]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.17334953, 51.61670267], [-127.92753044, 51.61670267], [-127.92753044, 51.73677458], [-128.17334953, 51.73677458], [-128.17334953, 51.61670267]]]}</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '10.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>oxygen, dissolvedOrganicCarbon, subSurfaceSalinity, subSurfaceTemperature, seaSurfaceHeight</t>
-        </is>
-      </c>
-      <c r="R64" t="inlineStr"/>
+          <t>other, invertebrateAbundanceAndDistribution</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>10.21966/kddh-gj22</t>
+        </is>
+      </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MW5xCIKrrtNHbrGqNTx</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWpwT0Z6RlAySHp6cU0</t>
         </is>
       </c>
       <c r="T64" t="inlineStr">
         <is>
-          <t>2022-02-01</t>
+          <t>2022-01-24</t>
         </is>
       </c>
       <c r="U64" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V64" t="n">
-        <v>2</v>
-      </c>
-      <c r="W64" t="inlineStr"/>
-      <c r="X64" t="inlineStr"/>
-      <c r="Y64" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="W64" t="n">
+        <v>0</v>
+      </c>
+      <c r="X64" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -7589,12 +7601,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
+          <t>0c864dea-998e-4a5e-94d3-c5fbda339eee</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>ca-cioos_87a845e3-e71a-43cc-a75f-ec6a3b812a0e</t>
+          <t>ca-cioos_41b0137d-6ac0-407d-a550-dd375475b2b0</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -7604,7 +7616,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Acoustic Doppler Current Profiler Time Series from Fixed Platform on the British Columbia Central Coast (Provisional)</t>
+          <t>Seafloor Observatory in Hyacinthe Bay, Quadra Island, British Columbia, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -7650,23 +7662,23 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.2, 51.61], [-128.6, 51.95], [-128.2, 52.04], [-127.8, 51.61], [-125.0, 50.12], [-125.2, 50.04], [-125.2, 50.04], [-125.2, 50.04], [-128.2, 51.61]]]}</t>
+          <t>{'type': 'Point', 'coordinates': [-125.22003, 50.11736]}</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>[{'max': '90.0', 'min': '0.0'}]</t>
+          <t>[{'max': '20.0', 'min': '10.0'}]</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>subSurfaceCurrents, subSurfaceTemperature, seaSurfaceHeight</t>
+          <t>oxygen, dissolvedOrganicCarbon, subSurfaceSalinity, subSurfaceTemperature, seaSurfaceHeight</t>
         </is>
       </c>
       <c r="R65" t="inlineStr"/>
       <c r="S65" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MsbCMOYj2L_7dgICnzw</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MW5xCIKrrtNHbrGqNTx</t>
         </is>
       </c>
       <c r="T65" t="inlineStr">
@@ -7676,11 +7688,11 @@
       </c>
       <c r="U65" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="V65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W65" t="inlineStr"/>
       <c r="X65" t="inlineStr"/>
@@ -7692,12 +7704,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>15f1d4a2-c82a-450c-a8f7-badb34b9c0dc</t>
+          <t>9c581481-f2ee-4353-b1ab-c5bf242945fe</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>ca-cioos_e09522d7-24f7-4c0e-afac-6cafd22a54f6</t>
+          <t>ca-cioos_87a845e3-e71a-43cc-a75f-ec6a3b812a0e</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -7707,7 +7719,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>High-resolution record of CO2 content from October 2013 to December 2018 measured in seawater entering the Alutiiq Pride Shellfish Hatchery in Seward, Alaska, USA</t>
+          <t>Acoustic Doppler Current Profiler Time Series from Fixed Platform on the British Columbia Central Coast (Provisional)</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -7730,7 +7742,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -7753,27 +7765,23 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-150.14476634, 59.68961051], [-148.42177964, 59.68961051], [-148.42177964, 60.2984757], [-150.14476634, 60.2984757], [-150.14476634, 59.68961051]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.2, 51.61], [-128.6, 51.95], [-128.2, 52.04], [-127.8, 51.61], [-125.0, 50.12], [-125.2, 50.04], [-125.2, 50.04], [-125.2, 50.04], [-128.2, 51.61]]]}</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '90.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
-        </is>
-      </c>
-      <c r="R66" t="inlineStr">
-        <is>
-          <t>10.21966/nkcy-8c07</t>
-        </is>
-      </c>
+          <t>subSurfaceCurrents, subSurfaceTemperature, seaSurfaceHeight</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr"/>
       <c r="S66" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVZUYVNsZXAyTXh5bnQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MsbCMOYj2L_7dgICnzw</t>
         </is>
       </c>
       <c r="T66" t="inlineStr">
@@ -7783,25 +7791,15 @@
       </c>
       <c r="U66" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="V66" t="n">
-        <v>6</v>
-      </c>
-      <c r="W66" t="n">
-        <v>0</v>
-      </c>
-      <c r="X66" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="Y66" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="W66" t="inlineStr"/>
+      <c r="X66" t="inlineStr"/>
+      <c r="Y66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -7809,12 +7807,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
+          <t>15f1d4a2-c82a-450c-a8f7-badb34b9c0dc</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>ca-cioos_4b5c0c20-2115-4986-bf56-237e360240bd</t>
+          <t>ca-cioos_e09522d7-24f7-4c0e-afac-6cafd22a54f6</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -7824,7 +7822,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018</t>
+          <t>High-resolution record of CO2 content from October 2013 to December 2018 measured in seawater entering the Alutiiq Pride Shellfish Hatchery in Seward, Alaska, USA</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -7842,7 +7840,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>Oceanography, Watersheds</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -7870,7 +7868,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.2, 51.64], [-127.9, 51.64], [-127.9, 51.74], [-128.2, 51.74], [-128.2, 51.64]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-150.14476634, 59.68961051], [-148.42177964, 59.68961051], [-148.42177964, 60.2984757], [-150.14476634, 60.2984757], [-150.14476634, 59.68961051]]]}</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
@@ -7880,43 +7878,43 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>nutrients, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
         <is>
-          <t>10.21966/n0h9-cq15</t>
+          <t>10.21966/nkcy-8c07</t>
         </is>
       </c>
       <c r="S67" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MuwHJS-RtHVqJmki_OG</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVZUYVNsZXAyTXh5bnQ</t>
         </is>
       </c>
       <c r="T67" t="inlineStr">
         <is>
-          <t>2022-02-02</t>
+          <t>2022-02-01</t>
         </is>
       </c>
       <c r="U67" t="inlineStr">
         <is>
-          <t>2025-01-30</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V67" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="W67" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X67" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="Y67" t="inlineStr">
         <is>
-          <t>[{'relationship': 'citations', 'id': '10.5194/bg-18-3029-2021', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/18/3029/2021/'}, {'relationship': 'parts', 'id': '10.5194/bg-2020-350', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/18/3029/2021/bg-18-3029-2021-discussion.html'}]</t>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -7926,12 +7924,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
+          <t>1a9a5aae-41ee-4272-a52e-6c37abedfbff</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>ca-cioos_a0ca5d26-b457-4726-97d4-ed0c8dd6cd99</t>
+          <t>ca-cioos_4b5c0c20-2115-4986-bf56-237e360240bd</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -7941,7 +7939,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Seascape connectivity data from a sub-tidal Zostera marina meadow, Choked Passage, Calvert Island, 2015</t>
+          <t>Freshwater and marine water quality (nutrients and carbon) - Calvert Island - 2014 to 2018</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -7959,7 +7957,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography, Watersheds</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -7987,7 +7985,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.2, 51.64], [-127.9, 51.64], [-127.9, 51.74], [-128.2, 51.74], [-128.2, 51.64]]]}</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
@@ -7997,17 +7995,17 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>other, seagrassCoverAndComposition</t>
+          <t>nutrients, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>10.21966/exy6-1k58</t>
+          <t>10.21966/n0h9-cq15</t>
         </is>
       </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUoydUo4NEl3VEtGdU0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MuwHJS-RtHVqJmki_OG</t>
         </is>
       </c>
       <c r="T68" t="inlineStr">
@@ -8017,23 +8015,23 @@
       </c>
       <c r="U68" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2025-01-30</t>
         </is>
       </c>
       <c r="V68" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="W68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X68" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="Y68" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'relationship': 'citations', 'id': '10.5194/bg-18-3029-2021', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/18/3029/2021/'}, {'relationship': 'parts', 'id': '10.5194/bg-2020-350', 'type': 'dois', 'status_code': 200, 'url': 'https://bg.copernicus.org/articles/18/3029/2021/bg-18-3029-2021-discussion.html'}]</t>
         </is>
       </c>
     </row>
@@ -8043,12 +8041,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>4becb6c2-ebdb-43f2-8f15-dee50aaa19d8</t>
+          <t>dd30b32a-2099-4909-838d-6ade9804381a</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>ca-cioos_fd5ada9a-5719-4ca1-89d2-17adb48d1493</t>
+          <t>ca-cioos_a0ca5d26-b457-4726-97d4-ed0c8dd6cd99</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -8058,7 +8056,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Eelgrass (Z. marina) extent at Gulf Islands National Park Reserve eelgrass monitoring sites (2017, 2018) v1.0.0</t>
+          <t>Seascape connectivity data from a sub-tidal Zostera marina meadow, Choked Passage, Calvert Island, 2015</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -8076,7 +8074,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Nearshore, Geospatial</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -8104,27 +8102,27 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-123.81789453, 48.48393505], [-122.96096027, 48.48393505], [-122.96096027, 49.05595865], [-123.81789453, 49.05595865], [-123.81789453, 48.48393505]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>[{'max': '100.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, seagrassCoverAndComposition</t>
         </is>
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>10.21966/t8hm-ge90</t>
+          <t>10.21966/exy6-1k58</t>
         </is>
       </c>
       <c r="S69" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBNZnZGekFJcFFDcm8</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUoydUo4NEl3VEtGdU0</t>
         </is>
       </c>
       <c r="T69" t="inlineStr">
@@ -8134,10 +8132,12 @@
       </c>
       <c r="U69" t="inlineStr">
         <is>
-          <t>2024-11-25</t>
-        </is>
-      </c>
-      <c r="V69" t="inlineStr"/>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="V69" t="n">
+        <v>9</v>
+      </c>
       <c r="W69" t="n">
         <v>0</v>
       </c>
@@ -8158,12 +8158,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>26186b9d-a292-43c4-aec6-e928aa52b002</t>
+          <t>4becb6c2-ebdb-43f2-8f15-dee50aaa19d8</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>ca-cioos_63765cc6-5730-4a28-9d96-3de38066312f</t>
+          <t>ca-cioos_fd5ada9a-5719-4ca1-89d2-17adb48d1493</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -8173,7 +8173,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>High-resolution record of surface seawater CO2 content from April 2016 to November 2017 collected in Hyacinthe Bay, British Columbia, Canada</t>
+          <t>Eelgrass (Z. marina) extent at Gulf Islands National Park Reserve eelgrass monitoring sites (2017, 2018) v1.0.0</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -8191,7 +8191,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore, Geospatial</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -8215,41 +8215,41 @@
         </is>
       </c>
       <c r="N70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.22364854812619, 50.116106505752896], [-125.22126674652097, 50.116106505752896], [-125.22126674652097, 50.11770256813347], [-125.22364854812619, 50.11770256813347], [-125.22364854812619, 50.116106505752896]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.81789453, 48.48393505], [-122.96096027, 48.48393505], [-122.96096027, 49.05595865], [-123.81789453, 49.05595865], [-123.81789453, 48.48393505]]]}</t>
         </is>
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '100.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>10.21966/1.614670</t>
+          <t>10.21966/t8hm-ge90</t>
         </is>
       </c>
       <c r="S70" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVpjRzlIZEFLbE9tSnA</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBNZnZGekFJcFFDcm8</t>
         </is>
       </c>
       <c r="T70" t="inlineStr">
         <is>
-          <t>2022-02-03</t>
+          <t>2022-02-02</t>
         </is>
       </c>
       <c r="U70" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2024-11-25</t>
         </is>
       </c>
       <c r="V70" t="inlineStr"/>
@@ -8273,12 +8273,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
+          <t>26186b9d-a292-43c4-aec6-e928aa52b002</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>ca-cioos_7c47472a-b16c-446c-89d5-eefa23e07922</t>
+          <t>ca-cioos_63765cc6-5730-4a28-9d96-3de38066312f</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -8288,7 +8288,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>High-resolution record of surface seawater CO2 content from November 2017 to June 2018 collected in Hyacinthe Bay, British Columbia, Canada</t>
+          <t>High-resolution record of surface seawater CO2 content from April 2016 to November 2017 collected in Hyacinthe Bay, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -8330,7 +8330,7 @@
         </is>
       </c>
       <c r="N71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
@@ -8349,12 +8349,12 @@
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>10.21966/1.715729</t>
+          <t>10.21966/1.614670</t>
         </is>
       </c>
       <c r="S71" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUhwbUdDUUlVTWtHYzE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVpjRzlIZEFLbE9tSnA</t>
         </is>
       </c>
       <c r="T71" t="inlineStr">
@@ -8364,12 +8364,10 @@
       </c>
       <c r="U71" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
-        </is>
-      </c>
-      <c r="V71" t="n">
-        <v>1</v>
-      </c>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr"/>
       <c r="W71" t="n">
         <v>0</v>
       </c>
@@ -8390,12 +8388,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
+          <t>f31f38bf-16bc-4136-8982-a2df5fefb3a0</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>ca-cioos_a72c43e2-5b4d-4d56-89d4-464b4c513710</t>
+          <t>ca-cioos_7c47472a-b16c-446c-89d5-eefa23e07922</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -8405,7 +8403,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by shellfish growers and partners in the northern Salish Sea from 2016 to 2018</t>
+          <t>High-resolution record of surface seawater CO2 content from November 2017 to June 2018 collected in Hyacinthe Bay, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -8451,7 +8449,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.57747949, 49.70969514], [-124.52984083, 49.70969514], [-124.52984083, 50.11496976], [-125.57747949, 50.11496976], [-125.57747949, 49.70969514]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.22364854812619, 50.116106505752896], [-125.22126674652097, 50.116106505752896], [-125.22126674652097, 50.11770256813347], [-125.22364854812619, 50.11770256813347], [-125.22364854812619, 50.116106505752896]]]}</t>
         </is>
       </c>
       <c r="P72" t="inlineStr">
@@ -8466,12 +8464,12 @@
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>10.21966/1.715756</t>
+          <t>10.21966/1.715729</t>
         </is>
       </c>
       <c r="S72" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWYwNjRsV2piMFJOR08</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUhwbUdDUUlVTWtHYzE</t>
         </is>
       </c>
       <c r="T72" t="inlineStr">
@@ -8481,7 +8479,7 @@
       </c>
       <c r="U72" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V72" t="n">
@@ -8507,12 +8505,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>6338c2fa-3d4d-42dc-9c91-31761365e11e</t>
+          <t>45983472-7627-4227-b312-079c2aeda7ef</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>ca-cioos_77a256cd-baf7-434e-9f62-53ba809e48cb</t>
+          <t>ca-cioos_a72c43e2-5b4d-4d56-89d4-464b4c513710</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -8522,7 +8520,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>High-resolution record of 8-m seawater CO2 content entering Fanny Bay Oysters in Baynes Sound, British Columbia, Canada from March 2017 to November 2017</t>
+          <t>Surface water CO2 parameters collected by shellfish growers and partners in the northern Salish Sea from 2016 to 2018</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -8564,11 +8562,11 @@
         </is>
       </c>
       <c r="N73" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.88983154296876, 49.44759314103575], [-124.70993041992188, 49.44759314103575], [-124.70993041992188, 49.56975910961884], [-124.88983154296876, 49.56975910961884], [-124.88983154296876, 49.44759314103575]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.57747949, 49.70969514], [-124.52984083, 49.70969514], [-124.52984083, 50.11496976], [-125.57747949, 50.11496976], [-125.57747949, 49.70969514]]]}</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
@@ -8583,22 +8581,22 @@
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>10.21966/1.622315</t>
+          <t>10.21966/1.715756</t>
         </is>
       </c>
       <c r="S73" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTV4aEZoVWsyRXpHWno</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWYwNjRsV2piMFJOR08</t>
         </is>
       </c>
       <c r="T73" t="inlineStr">
         <is>
-          <t>2022-02-04</t>
+          <t>2022-02-03</t>
         </is>
       </c>
       <c r="U73" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V73" t="n">
@@ -8624,12 +8622,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>d3ed88cb-4f38-4c2e-a966-3dd49c9cafec</t>
+          <t>6338c2fa-3d4d-42dc-9c91-31761365e11e</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ca-cioos_804b5b42-5550-4620-b789-7c2fe9572c03</t>
+          <t>ca-cioos_77a256cd-baf7-434e-9f62-53ba809e48cb</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -8639,7 +8637,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Zooplankton - Taxonomy – Northern Strait of Georgia, Discovery Islands, Johnstone Strait, and Queen Charlotte Strait – April to July 2015 and 2016</t>
+          <t>High-resolution record of 8-m seawater CO2 content entering Fanny Bay Oysters in Baynes Sound, British Columbia, Canada from March 2017 to November 2017</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -8662,7 +8660,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>underDevelopment</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -8681,45 +8679,45 @@
         </is>
       </c>
       <c r="N74" t="n">
+        <v>3</v>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.88983154296876, 49.44759314103575], [-124.70993041992188, 49.44759314103575], [-124.70993041992188, 49.56975910961884], [-124.88983154296876, 49.56975910961884], [-124.88983154296876, 49.44759314103575]]]}</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>other, inorganicCarbon</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>10.21966/1.622315</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTV4aEZoVWsyRXpHWno</t>
+        </is>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>2022-02-04</t>
+        </is>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>2024-07-23</t>
+        </is>
+      </c>
+      <c r="V74" t="n">
         <v>1</v>
-      </c>
-      <c r="O74" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.93452704, 49.56730131], [-124.18481219, 49.56730131], [-124.18481219, 50.90762515], [-126.93452704, 50.90762515], [-126.93452704, 49.56730131]]]}</t>
-        </is>
-      </c>
-      <c r="P74" t="inlineStr">
-        <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q74" t="inlineStr">
-        <is>
-          <t>other, zooplanktonBiomassAndDiversity</t>
-        </is>
-      </c>
-      <c r="R74" t="inlineStr">
-        <is>
-          <t>10.21966/bhqd-9361</t>
-        </is>
-      </c>
-      <c r="S74" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTZhamNPb0U3cThnR0o</t>
-        </is>
-      </c>
-      <c r="T74" t="inlineStr">
-        <is>
-          <t>2022-02-04</t>
-        </is>
-      </c>
-      <c r="U74" t="inlineStr">
-        <is>
-          <t>2024-07-23</t>
-        </is>
-      </c>
-      <c r="V74" t="n">
-        <v>5</v>
       </c>
       <c r="W74" t="n">
         <v>0</v>
@@ -8741,12 +8739,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>7f23d45b-b777-491c-b602-def5402d3d83</t>
+          <t>d3ed88cb-4f38-4c2e-a966-3dd49c9cafec</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_a0263680-f0d5-46d5-85ea-483fa58c74b6</t>
+          <t>ca-cioos_804b5b42-5550-4620-b789-7c2fe9572c03</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8756,7 +8754,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>High-resolution record of sea surface nitrate at Sentry Shoal in the Northern Strait of Georgia, British Columbia, Canada from 2015 to 2017.</t>
+          <t>Zooplankton - Taxonomy – Northern Strait of Georgia, Discovery Islands, Johnstone Strait, and Queen Charlotte Strait – April to July 2015 and 2016</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8798,11 +8796,11 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.2942704, 49.83702595], [-124.90571487, 49.83702595], [-124.90571487, 50.05976151], [-125.2942704, 50.05976151], [-125.2942704, 49.83702595]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.93452704, 49.56730131], [-124.18481219, 49.56730131], [-124.18481219, 50.90762515], [-126.93452704, 50.90762515], [-126.93452704, 49.56730131]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
@@ -8812,17 +8810,17 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>nutrients</t>
+          <t>other, zooplanktonBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/yk87-4x24</t>
+          <t>10.21966/bhqd-9361</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTZ1QmZ1a3ZiZWEwM24</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTZhamNPb0U3cThnR0o</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8832,12 +8830,10 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
-        </is>
-      </c>
-      <c r="V75" t="n">
-        <v>4</v>
-      </c>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="V75" t="inlineStr"/>
       <c r="W75" t="n">
         <v>0</v>
       </c>
@@ -8858,12 +8854,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>7f23d45b-b777-491c-b602-def5402d3d83</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_a0263680-f0d5-46d5-85ea-483fa58c74b6</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8873,7 +8869,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>High-resolution record of sea surface nitrate at Sentry Shoal in the Northern Strait of Georgia, British Columbia, Canada from 2015 to 2017.</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8889,10 +8885,14 @@
       <c r="H76" t="b">
         <v>0</v>
       </c>
-      <c r="I76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Oceanography</t>
+        </is>
+      </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>underDevelopment</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -8915,28 +8915,32 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.2942704, 49.83702595], [-124.90571487, 49.83702595], [-124.90571487, 50.05976151], [-125.2942704, 50.05976151], [-125.2942704, 49.83702595]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R76" t="inlineStr"/>
+          <t>nutrients</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>10.21966/yk87-4x24</t>
+        </is>
+      </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTZ1QmZ1a3ZiZWEwM24</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
         <is>
-          <t>2022-03-01</t>
+          <t>2022-02-04</t>
         </is>
       </c>
       <c r="U76" t="inlineStr">
@@ -8947,9 +8951,19 @@
       <c r="V76" t="n">
         <v>4</v>
       </c>
-      <c r="W76" t="inlineStr"/>
-      <c r="X76" t="inlineStr"/>
-      <c r="Y76" t="inlineStr"/>
+      <c r="W76" t="n">
+        <v>0</v>
+      </c>
+      <c r="X76" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Y76" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -9060,12 +9074,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ca-cioos_62de21ed-90fb-422a-9c55-29c513a00f95</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -9075,7 +9089,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Kilbella River Estuary LiDAR Survey - 2019 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -9091,11 +9105,7 @@
       <c r="H78" t="b">
         <v>0</v>
       </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>Airborne Coastal Observatory</t>
-        </is>
-      </c>
+      <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr">
         <is>
           <t>completed</t>
@@ -9121,12 +9131,12 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 51.72], [-127.3, 51.72], [-127.3, 51.74], [-127.4, 51.74], [-127.4, 51.72]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -9137,7 +9147,7 @@
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6CPeL2BfoPN85rGFk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T78" t="inlineStr">
@@ -9151,7 +9161,7 @@
         </is>
       </c>
       <c r="V78" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr"/>
@@ -9163,12 +9173,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>b5ee0615-c04d-462e-8199-f611bc6370ce</t>
+          <t>e3205958-52b4-4c42-a02d-34d713a20a53</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>ca-cioos_95bee6a0-ae38-4427-b5b2-5cc5835df70d</t>
+          <t>ca-cioos_62de21ed-90fb-422a-9c55-29c513a00f95</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -9178,7 +9188,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>North Vancouver Island Survey - 2019 - Airborne Coastal Observatory</t>
+          <t>Kilbella River Estuary LiDAR Survey - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -9194,7 +9204,11 @@
       <c r="H79" t="b">
         <v>0</v>
       </c>
-      <c r="I79" t="inlineStr"/>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory</t>
+        </is>
+      </c>
       <c r="J79" t="inlineStr">
         <is>
           <t>completed</t>
@@ -9220,12 +9234,12 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.3, 50.33], [-127.6, 50.33], [-127.6, 50.63], [-128.3, 50.63], [-128.3, 50.33]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 51.72], [-127.3, 51.72], [-127.3, 51.74], [-127.4, 51.74], [-127.4, 51.72]]]}</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">
@@ -9236,7 +9250,7 @@
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6hTZuLZ6h5NLfVXzz</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6CPeL2BfoPN85rGFk</t>
         </is>
       </c>
       <c r="T79" t="inlineStr">
@@ -9250,7 +9264,7 @@
         </is>
       </c>
       <c r="V79" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W79" t="inlineStr"/>
       <c r="X79" t="inlineStr"/>
@@ -9262,12 +9276,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>727b8863-91cc-4765-b0c0-80cb74b11182</t>
+          <t>b5ee0615-c04d-462e-8199-f611bc6370ce</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>ca-cioos_a60a0468-3f56-4f22-abd4-5268fcfb9744</t>
+          <t>ca-cioos_95bee6a0-ae38-4427-b5b2-5cc5835df70d</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -9277,7 +9291,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Owikeno Basin LiDAR Survey - 2019 - Airborne Coastal Observatory</t>
+          <t>North Vancouver Island Survey - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -9319,12 +9333,12 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.3, 51.46], [-125.9, 51.46], [-125.9, 51.92], [-127.3, 51.92], [-127.3, 51.46]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.3, 50.33], [-127.6, 50.33], [-127.6, 50.63], [-128.3, 50.63], [-128.3, 50.33]]]}</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>[{'max': '2500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q80" t="inlineStr">
@@ -9335,7 +9349,7 @@
       <c r="R80" t="inlineStr"/>
       <c r="S80" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MjBOaZ2eyXo9wQ38kdy</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6hTZuLZ6h5NLfVXzz</t>
         </is>
       </c>
       <c r="T80" t="inlineStr">
@@ -9361,12 +9375,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>5b78f1a7-6adb-4610-9ebe-019c3da65ae8</t>
+          <t>727b8863-91cc-4765-b0c0-80cb74b11182</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ca-cioos_bb59cb9e-887a-40a3-b41a-f4a5b2263ce6</t>
+          <t>ca-cioos_a60a0468-3f56-4f22-abd4-5268fcfb9744</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -9376,7 +9390,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Fountain Valley LiDAR Data - 2019 &amp; 2020 - Hakai Airborne Coastal Observatory - British Columbia - Canada</t>
+          <t>Owikeno Basin LiDAR Survey - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -9418,12 +9432,12 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-122.0, 50.56], [-121.7, 50.56], [-121.7, 50.8], [-122.0, 50.8], [-122.0, 50.56]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.3, 51.46], [-125.9, 51.46], [-125.9, 51.92], [-127.3, 51.92], [-127.3, 51.46]]]}</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>[{'max': '1500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr">
@@ -9434,7 +9448,7 @@
       <c r="R81" t="inlineStr"/>
       <c r="S81" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MmUnbGWVNvtiQAsYVPj</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MjBOaZ2eyXo9wQ38kdy</t>
         </is>
       </c>
       <c r="T81" t="inlineStr">
@@ -9460,12 +9474,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
+          <t>5b78f1a7-6adb-4610-9ebe-019c3da65ae8</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
+          <t>ca-cioos_bb59cb9e-887a-40a3-b41a-f4a5b2263ce6</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -9475,7 +9489,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
+          <t>Fountain Valley LiDAR Data - 2019 &amp; 2020 - Hakai Airborne Coastal Observatory - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -9491,11 +9505,7 @@
       <c r="H82" t="b">
         <v>0</v>
       </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>Airborne Coastal Observatory</t>
-        </is>
-      </c>
+      <c r="I82" t="inlineStr"/>
       <c r="J82" t="inlineStr">
         <is>
           <t>completed</t>
@@ -9521,12 +9531,12 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-122.0, 50.56], [-121.7, 50.56], [-121.7, 50.8], [-122.0, 50.8], [-122.0, 50.56]]]}</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>[{'max': '150.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
@@ -9534,14 +9544,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R82" t="inlineStr">
-        <is>
-          <t>10.21966/wfcv-n753</t>
-        </is>
-      </c>
+      <c r="R82" t="inlineStr"/>
       <c r="S82" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MmUnbGWVNvtiQAsYVPj</t>
         </is>
       </c>
       <c r="T82" t="inlineStr">
@@ -9555,21 +9561,11 @@
         </is>
       </c>
       <c r="V82" t="n">
-        <v>3</v>
-      </c>
-      <c r="W82" t="n">
-        <v>0</v>
-      </c>
-      <c r="X82" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="Y82" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="W82" t="inlineStr"/>
+      <c r="X82" t="inlineStr"/>
+      <c r="Y82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -9577,12 +9573,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
+          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
+          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -9592,7 +9588,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
+          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -9610,7 +9606,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -9638,12 +9634,12 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
         </is>
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '150.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr">
@@ -9653,12 +9649,12 @@
       </c>
       <c r="R83" t="inlineStr">
         <is>
-          <t>10.21966/eysg-7a26</t>
+          <t>10.21966/wfcv-n753</t>
         </is>
       </c>
       <c r="S83" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
         </is>
       </c>
       <c r="T83" t="inlineStr">
@@ -9694,12 +9690,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>8d3f619f-e3e5-44a7-8b35-7e4ed1e6af31</t>
+          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>ca-cioos_d2e83e40-9e95-4a47-a899-b37c744be3ab</t>
+          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -9709,7 +9705,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Fin Island &amp; K'yel - 2020 - Airborne Coastal Observatory Data</t>
+          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -9725,7 +9721,11 @@
       <c r="H84" t="b">
         <v>0</v>
       </c>
-      <c r="I84" t="inlineStr"/>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Geospatial, Airborne Coastal Observatory</t>
+        </is>
+      </c>
       <c r="J84" t="inlineStr">
         <is>
           <t>completed</t>
@@ -9751,7 +9751,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.4, 53.03], [-129.1, 53.03], [-129.1, 53.29], [-129.4, 53.29], [-129.4, 53.03]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
         </is>
       </c>
       <c r="P84" t="inlineStr">
@@ -9764,10 +9764,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R84" t="inlineStr"/>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>10.21966/eysg-7a26</t>
+        </is>
+      </c>
       <c r="S84" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNm5cwomXVNI6vWU-R</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
         </is>
       </c>
       <c r="T84" t="inlineStr">
@@ -9781,11 +9785,21 @@
         </is>
       </c>
       <c r="V84" t="n">
-        <v>4</v>
-      </c>
-      <c r="W84" t="inlineStr"/>
-      <c r="X84" t="inlineStr"/>
-      <c r="Y84" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="W84" t="n">
+        <v>0</v>
+      </c>
+      <c r="X84" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Y84" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -9793,12 +9807,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>826d8228-baab-4191-82de-44701cd93806</t>
+          <t>8d3f619f-e3e5-44a7-8b35-7e4ed1e6af31</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>ca-cioos_e0c768fc-5c37-455f-b2a3-604f766f4148</t>
+          <t>ca-cioos_d2e83e40-9e95-4a47-a899-b37c744be3ab</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -9808,7 +9822,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Nanwakolas Watershed Surveys - Knight Inlet - 2019 - Hakai Airborne Coastal Observatory</t>
+          <t>Fin Island &amp; K'yel - 2020 - Airborne Coastal Observatory Data</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -9850,12 +9864,12 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.1, 50.54], [-125.3, 50.54], [-125.3, 51.02], [-126.1, 51.02], [-126.1, 50.54]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.4, 53.03], [-129.1, 53.03], [-129.1, 53.29], [-129.4, 53.29], [-129.4, 53.03]]]}</t>
         </is>
       </c>
       <c r="P85" t="inlineStr">
         <is>
-          <t>[{'max': '1500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q85" t="inlineStr">
@@ -9866,7 +9880,7 @@
       <c r="R85" t="inlineStr"/>
       <c r="S85" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkEoax-I-IalULFPmu9</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNm5cwomXVNI6vWU-R</t>
         </is>
       </c>
       <c r="T85" t="inlineStr">
@@ -9892,12 +9906,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>571ef4fa-eda3-4e67-baae-2e9b5e598f56</t>
+          <t>826d8228-baab-4191-82de-44701cd93806</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>ca-cioos_2a92ca16-f5c6-4362-acea-6bb5117b8d65</t>
+          <t>ca-cioos_e0c768fc-5c37-455f-b2a3-604f766f4148</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -9907,7 +9921,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Google Earth Engine Kelp Tool - Central Coast Output - Version 1.0.0</t>
+          <t>Nanwakolas Watershed Surveys - Knight Inlet - 2019 - Hakai Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -9923,11 +9937,7 @@
       <c r="H86" t="b">
         <v>0</v>
       </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>Geospatial</t>
-        </is>
-      </c>
+      <c r="I86" t="inlineStr"/>
       <c r="J86" t="inlineStr">
         <is>
           <t>completed</t>
@@ -9953,12 +9963,12 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-130.35642493, 50.22213452], [-126.18162025, 50.22213452], [-126.18162025, 52.9911972], [-130.35642493, 52.9911972], [-130.35642493, 50.22213452]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.1, 50.54], [-125.3, 50.54], [-125.3, 51.02], [-126.1, 51.02], [-126.1, 50.54]]]}</t>
         </is>
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q86" t="inlineStr">
@@ -9969,12 +9979,12 @@
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFUcWNIVGxwZEVLNTE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkEoax-I-IalULFPmu9</t>
         </is>
       </c>
       <c r="T86" t="inlineStr">
         <is>
-          <t>2022-03-02</t>
+          <t>2022-03-01</t>
         </is>
       </c>
       <c r="U86" t="inlineStr">
@@ -10112,12 +10122,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
+          <t>571ef4fa-eda3-4e67-baae-2e9b5e598f56</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>ca-cioos_5c13b300-e172-4010-a6d8-7586b68a3a96</t>
+          <t>ca-cioos_2a92ca16-f5c6-4362-acea-6bb5117b8d65</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -10127,7 +10137,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Kelp extent for the McNaughton Group Islands (2017), Manley Island (2017), and Serpent Group Islands (2016), British Columbia, Canada</t>
+          <t>Google Earth Engine Kelp Tool - Central Coast Output - Version 1.0.0</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -10145,7 +10155,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -10169,11 +10179,11 @@
         </is>
       </c>
       <c r="N88" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.30122253, 51.7689035], [-128.05512885, 51.7689035], [-128.05512885, 51.98187882], [-128.30122253, 51.98187882], [-128.30122253, 51.7689035]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-130.35642493, 50.22213452], [-126.18162025, 50.22213452], [-126.18162025, 52.9911972], [-130.35642493, 52.9911972], [-130.35642493, 50.22213452]]]}</t>
         </is>
       </c>
       <c r="P88" t="inlineStr">
@@ -10183,17 +10193,13 @@
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>other, macroalgalCanopyCoverAndComposition</t>
-        </is>
-      </c>
-      <c r="R88" t="inlineStr">
-        <is>
-          <t>10.21966/82bd-ks94</t>
-        </is>
-      </c>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr"/>
       <c r="S88" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFIWmZWeEE0RkZrZVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFUcWNIVGxwZEVLNTE</t>
         </is>
       </c>
       <c r="T88" t="inlineStr">
@@ -10209,19 +10215,9 @@
       <c r="V88" t="n">
         <v>4</v>
       </c>
-      <c r="W88" t="n">
-        <v>0</v>
-      </c>
-      <c r="X88" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="Y88" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="W88" t="inlineStr"/>
+      <c r="X88" t="inlineStr"/>
+      <c r="Y88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -10229,12 +10225,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>1ad9809b-16a0-44f4-abc8-a1474b728c15</t>
+          <t>c8f6fd7c-7c63-440b-b69a-bd0df3abfd26</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>ca-cioos_5e4f925a-9cf2-4e33-ae22-75c5b326ce6c</t>
+          <t>ca-cioos_5c13b300-e172-4010-a6d8-7586b68a3a96</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -10244,7 +10240,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Eelgrass (Z. marina) extent at sites along the Central Coast, British Columbia</t>
+          <t>Kelp extent for the McNaughton Group Islands (2017), Manley Island (2017), and Serpent Group Islands (2016), British Columbia, Canada</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -10262,7 +10258,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Nearshore, Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -10286,11 +10282,11 @@
         </is>
       </c>
       <c r="N89" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.65354407, 51.37817421], [-127.69773286, 51.37817421], [-127.69773286, 52.1127963], [-128.65354407, 52.1127963], [-128.65354407, 51.37817421]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.30122253, 51.7689035], [-128.05512885, 51.7689035], [-128.05512885, 51.98187882], [-128.30122253, 51.98187882], [-128.30122253, 51.7689035]]]}</t>
         </is>
       </c>
       <c r="P89" t="inlineStr">
@@ -10300,17 +10296,17 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, macroalgalCanopyCoverAndComposition</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
         <is>
-          <t>10.21966/03pw-2190</t>
+          <t>10.21966/82bd-ks94</t>
         </is>
       </c>
       <c r="S89" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTA3NnQ0NnRiemVLSFU</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFIWmZWeEE0RkZrZVc</t>
         </is>
       </c>
       <c r="T89" t="inlineStr">
@@ -11916,7 +11912,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>underDevelopment</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -11965,11 +11961,11 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="V104" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W104" t="inlineStr"/>
       <c r="X104" t="inlineStr"/>
@@ -15087,12 +15083,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -15102,7 +15098,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada. Version 1.0.</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -15120,7 +15116,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -15138,37 +15134,33 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M133" t="inlineStr">
-        <is>
-          <t>University of British Columbia</t>
-        </is>
-      </c>
+      <c r="M133" t="inlineStr"/>
       <c r="N133" t="n">
         <v>1</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R133" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S133" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T133" t="inlineStr">
@@ -15182,7 +15174,7 @@
         </is>
       </c>
       <c r="V133" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="W133" t="n">
         <v>0</v>
@@ -15204,12 +15196,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -15219,7 +15211,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada. Version 1.0.</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -15237,7 +15229,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -15255,33 +15247,37 @@
           <t>dataset</t>
         </is>
       </c>
-      <c r="M134" t="inlineStr"/>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>University of British Columbia</t>
+        </is>
+      </c>
       <c r="N134" t="n">
         <v>1</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S134" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T134" t="inlineStr">
@@ -15295,7 +15291,7 @@
         </is>
       </c>
       <c r="V134" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="W134" t="n">
         <v>0</v>
@@ -21552,7 +21548,9 @@
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="V188" t="inlineStr"/>
+      <c r="V188" t="n">
+        <v>1</v>
+      </c>
       <c r="W188" t="n">
         <v>0</v>
       </c>

</xml_diff>